<commit_message>
第4轮评测 - `surveykit export logs --verbose --output output/。
</commit_message>
<xml_diff>
--- a/output/完成率报告.xlsx
+++ b/output/完成率报告.xlsx
@@ -425,40 +425,45 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>问卷</t>
+          <t>survey</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>题目</t>
+          <t>column</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>总题数</t>
+          <t>completion_rate</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>已答题数</t>
+          <t>total_count</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>完成率</t>
+          <t>answered_count</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>passed</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>学生调查</t>
+          <t>完整测试</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -467,19 +472,22 @@
         </is>
       </c>
       <c r="C2" t="n">
+        <v>0.8333</v>
+      </c>
+      <c r="D2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E2" t="n">
         <v>10</v>
       </c>
-      <c r="D2" t="n">
-        <v>8</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0.8</v>
+      <c r="F2" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>学生调查</t>
+          <t>完整测试</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -488,19 +496,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>10</v>
+        <v>0.75</v>
       </c>
       <c r="D3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E3" t="n">
         <v>9</v>
       </c>
-      <c r="E3" t="n">
-        <v>0.9</v>
+      <c r="F3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>学生调查</t>
+          <t>完整测试</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -509,19 +520,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>10</v>
+        <v>0.9167</v>
       </c>
       <c r="D4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9</v>
+        <v>11</v>
+      </c>
+      <c r="F4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>学生调查</t>
+          <t>完整测试</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -530,19 +544,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>10</v>
+        <v>0.75</v>
       </c>
       <c r="D5" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>9</v>
+      </c>
+      <c r="F5" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>学生调查</t>
+          <t>完整测试</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -551,19 +568,22 @@
         </is>
       </c>
       <c r="C6" t="n">
+        <v>0.8333</v>
+      </c>
+      <c r="D6" t="n">
+        <v>12</v>
+      </c>
+      <c r="E6" t="n">
         <v>10</v>
       </c>
-      <c r="D6" t="n">
-        <v>9</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.9</v>
+      <c r="F6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>学生调查</t>
+          <t>完整测试</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -572,19 +592,22 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>10</v>
+        <v>0.6667</v>
       </c>
       <c r="D7" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E7" t="n">
-        <v>0.9</v>
+        <v>8</v>
+      </c>
+      <c r="F7" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>学生调查</t>
+          <t>完整测试</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -593,12 +616,15 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E8" t="n">
+        <v>12</v>
+      </c>
+      <c r="F8" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>